<commit_message>
feat: add detailed voter list column to standings Excel sheet and history registry
</commit_message>
<xml_diff>
--- a/.gemini/01_YOURVISION/09_CHARTS/YV_AllMix_VibeShift_2026_Recalculated_Standings.xlsx
+++ b/.gemini/01_YOURVISION/09_CHARTS/YV_AllMix_VibeShift_2026_Recalculated_Standings.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -504,6 +504,7 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="120" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -557,6 +558,11 @@
           <t>Статус</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Список проголосовавших</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -597,6 +603,11 @@
           <t>🏆 ПОБЕДА</t>
         </is>
       </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>GLN (1), levdanskiy (2), Туз Буби (2), Ильдус (5), Jane Marduk (5), Linh (6), ТЁМА С. 🦂 (8), Imants (10), Елена (11)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="5" t="n">
@@ -637,6 +648,11 @@
           <t>HIT 🔥</t>
         </is>
       </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Imants (1), Linh (1), Елена (3), ТЁМА С. 🦂 (3), Туз Буби (3), levdanskiy (6), Ильдус (12)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -677,6 +693,11 @@
           <t>HIT 🔥</t>
         </is>
       </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>PVL (1), Туз Буби (1), Jane Marduk (1), Елена (5), ТЁМА С. 🦂 (5), Ильдус (8), Linh (11)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="n">
@@ -717,6 +738,11 @@
           <t>HIT 🔥</t>
         </is>
       </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>PVL (2), Ильдус (3), levdanskiy (5), Елена (6), Jane Marduk (7), Туз Буби (8), Linh (9), Imants (11), GLN (12)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -757,6 +783,11 @@
           <t>HIT 🔥</t>
         </is>
       </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>ТЁМА С. 🦂 (1), Linh (4), Imants (5), GLN (5), Ильдус (7), Туз Буби (9), PVL (10)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="5" t="n">
@@ -797,6 +828,11 @@
           <t>HIT 🔥</t>
         </is>
       </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Елена (1), Linh (3), Jane Marduk (3), ТЁМА С. 🦂 (4), levdanskiy (4)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -837,6 +873,11 @@
           <t>TOP-10</t>
         </is>
       </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Елена (2), PVL (5), Imants (6), GLN (6), Linh (7), Jane Marduk (10), levdanskiy (11), Туз Буби (11)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="n">
@@ -877,6 +918,11 @@
           <t>TOP-10</t>
         </is>
       </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>GLN (2), Linh (5), ТЁМА С. 🦂 (6), Jane Marduk (6), levdanskiy (7), Туз Буби (10), Imants (12)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -917,6 +963,11 @@
           <t>TOP-10</t>
         </is>
       </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>levdanskiy (1), Елена (4), PVL (4), Imants (7), GLN (9), Jane Marduk (12)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="5" t="n">
@@ -957,6 +1008,11 @@
           <t>TOP-10</t>
         </is>
       </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Ильдус (1), Jane Marduk (2), Туз Буби (5), PVL (6), ТЁМА С. 🦂 (12)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -997,6 +1053,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>GLN (3), Туз Буби (4), PVL (7), levdanskiy (8), Jane Marduk (8), Елена (10)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="5" t="n">
@@ -1037,6 +1098,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>PVL (3), Туз Буби (7), Imants (8), Елена (9), ТЁМА С. 🦂 (9), Ильдус (10), GLN (11), Jane Marduk (11)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -1077,6 +1143,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>levdanskiy (3), Jane Marduk (4), Ильдус (6), Imants (9), ТЁМА С. 🦂 (10)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="5" t="n">
@@ -1117,6 +1188,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>ТЁМА С. 🦂 (2), Ильдус (4), Туз Буби (6), PVL (11)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -1157,6 +1233,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Ильдус (2), Imants (3), GLN (10), Linh (10), Елена (12)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="5" t="n">
@@ -1197,6 +1278,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>Linh (2), Imants (4), Ильдус (9), Jane Marduk (9)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -1237,6 +1323,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Imants (2), GLN (8), Linh (8), levdanskiy (10), Ильдус (11), PVL (12)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="5" t="n">
@@ -1277,6 +1368,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>ТЁМА С. 🦂 (7), GLN (7), Елена (8), PVL (8), levdanskiy (12)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -1317,6 +1413,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>GLN (4), PVL (9), Туз Буби (12)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="5" t="n">
@@ -1355,6 +1456,11 @@
       <c r="J21" s="7" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>Елена (7), levdanskiy (9), ТЁМА С. 🦂 (11), Linh (12)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: upgrade Excel sheet to a premium 3-sheet workbook with KPI Dashboard
</commit_message>
<xml_diff>
--- a/.gemini/01_YOURVISION/09_CHARTS/YV_AllMix_VibeShift_2026_Recalculated_Standings.xlsx
+++ b/.gemini/01_YOURVISION/09_CHARTS/YV_AllMix_VibeShift_2026_Recalculated_Standings.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Итоговая таблица" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Матрица голосов" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Панель управления" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Итоговая таблица" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Матрица голосов" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +19,37 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -42,12 +67,18 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F4F7"/>
+        <bgColor rgb="00F2F4F7"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -63,8 +94,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-        <bgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00F9FAFB"/>
+        <bgColor rgb="00F9FAFB"/>
       </patternFill>
     </fill>
     <fill>
@@ -74,13 +105,64 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="8">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001F4E78"/>
+      </left>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001F4E78"/>
+      </left>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001F4E78"/>
+      </left>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -100,30 +182,55 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -491,6 +598,515 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="37" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2" ht="30" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>🎼 YOURVISION CHARTS — ALLMIX: VIBE SHIFT 2026</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>ПОБЕДИТЕЛЬ РАУНДА</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="8" t="n"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>УЧАСТНИКИ ЖЮРИ</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>ХИТ-ТРЕКИ (HIT 🔥)</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>САМЫЙ ВЫСОКИЙ РЕЙТИНГ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Linda &amp; Pete — Liekinheitin (72б)</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>10 человек (120 оценок)</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>6 композиций</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Sal Da Vinci (8.3/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>🏆 КУБОК СТРАН (COUNTRY CUP)</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>⭐ ВЫБОР ЖЮРИ (JURY TOP FAVORITES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Место</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Страна / Регион</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Очки (Hit-Maker)</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Член жюри</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Любимый трек (1-е место)</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>Исполнитель</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>США 🇺🇸</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>223</v>
+      </c>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>GLN</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>«Liekinheitin»</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>Linda Lampenius &amp; Pete Parkkonen</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Россия 🇷🇺</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>189</v>
+      </c>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>Imants</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>«I Knew It, I Knew You»</t>
+        </is>
+      </c>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Южная Корея 🇰🇷</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>123</v>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Jane Marduk</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>«JUMP»</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>BLACKPINK</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Финляндия 🇫🇮</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>72</v>
+      </c>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>Linh</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>«I Knew It, I Knew You»</t>
+        </is>
+      </c>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Италия 🇮🇹</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>53</v>
+      </c>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>PVL</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
+          <t>«JUMP»</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>BLACKPINK</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Румыния 🇷🇴</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>44</v>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>levdanskiy</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>«KARMA»</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>Егор Крид, ARTIK &amp; ASTI</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>Швеция 🇸🇪</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>36</v>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Елена</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
+        <is>
+          <t>«Per sempre sì»</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t>Sal Da Vinci</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>Великобритания 🇬🇧</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>29</v>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>Ильдус</t>
+        </is>
+      </c>
+      <c r="G16" s="17" t="inlineStr">
+        <is>
+          <t>«PINKY UP»</t>
+        </is>
+      </c>
+      <c r="H16" s="17" t="inlineStr">
+        <is>
+          <t>KATSEYE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>Беларусь 🇧🇾</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>28</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>ТЁМА С. 🦂</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>«drop dead»</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>Болгария 🇧🇬</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>Туз Буби</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="inlineStr">
+        <is>
+          <t>«JUMP»</t>
+        </is>
+      </c>
+      <c r="H18" s="17" t="inlineStr">
+        <is>
+          <t>BLACKPINK</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21">
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>📊 ОБЩАЯ СТАТИСТИКА РАУНДА</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Всего номинировано треков</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>Сумма линейных баллов жюри</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Сумма прогрессивных баллов Hit-Maker</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Средняя вовлечённость жюри</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>61.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Средний рейтинг трека по шкале 10</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>5.13/10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="B2:K2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -508,957 +1124,957 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Новое место</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Исполнитель</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Песня</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Старое место</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Старые баллы (Линейные)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Новые баллы (Hit-Maker)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Голоса жюри</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Охват (%)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Средний рейтинг</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>Список проголосовавших</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Linda Lampenius &amp; Pete Parkkonen</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
         <is>
           <t>Liekinheitin</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="19" t="n">
         <v>67</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="12" t="n">
         <v>72</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="19" t="inlineStr">
         <is>
           <t>90%</t>
         </is>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="19" t="n">
         <v>6.2</v>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="19" t="inlineStr">
         <is>
           <t>🏆 ПОБЕДА</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="14" t="inlineStr">
         <is>
           <t>GLN (1), levdanskiy (2), Туз Буби (2), Ильдус (5), Jane Marduk (5), Linh (6), ТЁМА С. 🦂 (8), Imants (10), Елена (11)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>Taylor Swift</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>I Knew It, I Knew You</t>
         </is>
       </c>
-      <c r="D3" s="7" t="n">
+      <c r="D3" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="7" t="n">
+      <c r="E3" s="18" t="n">
         <v>62</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="15" t="n">
         <v>68</v>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="G3" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr">
         <is>
           <t>70%</t>
         </is>
       </c>
-      <c r="I3" s="7" t="n">
+      <c r="I3" s="18" t="n">
         <v>7.38</v>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="J3" s="18" t="inlineStr">
         <is>
           <t>HIT 🔥</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="K3" s="17" t="inlineStr">
         <is>
           <t>Imants (1), Linh (1), Елена (3), ТЁМА С. 🦂 (3), Туз Буби (3), levdanskiy (6), Ильдус (12)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>BLACKPINK</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>JUMP</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="19" t="n">
         <v>59</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="12" t="n">
         <v>68</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="19" t="inlineStr">
         <is>
           <t>70%</t>
         </is>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="19" t="n">
         <v>7.02</v>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="19" t="inlineStr">
         <is>
           <t>HIT 🔥</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="14" t="inlineStr">
         <is>
           <t>PVL (1), Туз Буби (1), Jane Marduk (1), Елена (5), ТЁМА С. 🦂 (5), Ильдус (8), Linh (11)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>BTS</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>SWIM</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="18" t="n">
         <v>54</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="18" t="inlineStr">
         <is>
           <t>90%</t>
         </is>
       </c>
-      <c r="I5" s="7" t="n">
+      <c r="I5" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="J5" s="18" t="inlineStr">
         <is>
           <t>HIT 🔥</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="K5" s="17" t="inlineStr">
         <is>
           <t>PVL (2), Ильдус (3), levdanskiy (5), Елена (6), Jane Marduk (7), Туз Буби (8), Linh (9), Imants (11), GLN (12)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>Olivia Rodrigo</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>drop dead</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="19" t="n">
         <v>50</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="12" t="n">
         <v>53</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="19" t="inlineStr">
         <is>
           <t>70%</t>
         </is>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="19" t="n">
         <v>5.95</v>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="19" t="inlineStr">
         <is>
           <t>HIT 🔥</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K6" s="14" t="inlineStr">
         <is>
           <t>ТЁМА С. 🦂 (1), Linh (4), Imants (5), GLN (5), Ильдус (7), Туз Буби (9), PVL (10)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Sal Da Vinci</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>Per sempre sì</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G7" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="18" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
       </c>
-      <c r="I7" s="7" t="n">
+      <c r="I7" s="18" t="n">
         <v>8.33</v>
       </c>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="J7" s="18" t="inlineStr">
         <is>
           <t>HIT 🔥</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="K7" s="17" t="inlineStr">
         <is>
           <t>Елена (1), Linh (3), Jane Marduk (3), ТЁМА С. 🦂 (4), levdanskiy (4)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>By Индия, Xcho, МОТ</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Шадэ</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="19" t="n">
         <v>46</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="12" t="n">
         <v>47</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="19" t="inlineStr">
         <is>
           <t>80%</t>
         </is>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="I8" s="19" t="n">
         <v>4.79</v>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="19" t="inlineStr">
         <is>
           <t>TOP-10</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K8" s="14" t="inlineStr">
         <is>
           <t>Елена (2), PVL (5), Imants (6), GLN (6), Linh (7), Jane Marduk (10), levdanskiy (11), Туз Буби (11)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Alexandra Căpitănescu</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>Choke Me</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="18" t="n">
         <v>43</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="G9" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="18" t="inlineStr">
         <is>
           <t>70%</t>
         </is>
       </c>
-      <c r="I9" s="7" t="n">
+      <c r="I9" s="18" t="n">
         <v>5.12</v>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J9" s="18" t="inlineStr">
         <is>
           <t>TOP-10</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>GLN (2), Linh (5), ТЁМА С. 🦂 (6), Jane Marduk (6), levdanskiy (7), Туз Буби (10), Imants (12)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Егор Крид, ARTIK &amp; ASTI</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>KARMA</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="19" t="n">
         <v>41</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="12" t="n">
         <v>44</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="G10" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="19" t="inlineStr">
         <is>
           <t>60%</t>
         </is>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="I10" s="19" t="n">
         <v>5.69</v>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="19" t="inlineStr">
         <is>
           <t>TOP-10</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K10" s="14" t="inlineStr">
         <is>
           <t>levdanskiy (1), Елена (4), PVL (4), Imants (7), GLN (9), Jane Marduk (12)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>KATSEYE</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>PINKY UP</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="18" t="n">
         <v>39</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="15" t="n">
         <v>43</v>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="G11" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" s="18" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
       </c>
-      <c r="I11" s="7" t="n">
+      <c r="I11" s="18" t="n">
         <v>6.5</v>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="J11" s="18" t="inlineStr">
         <is>
           <t>TOP-10</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>Ильдус (1), Jane Marduk (2), Туз Буби (5), PVL (6), ТЁМА С. 🦂 (12)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>BEARWOLF</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Феникс</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="19" t="n">
         <v>11</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="19" t="n">
         <v>38</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="12" t="n">
         <v>38</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="G12" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="19" t="inlineStr">
         <is>
           <t>60%</t>
         </is>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="I12" s="19" t="n">
         <v>5.28</v>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" s="19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K12" s="14" t="inlineStr">
         <is>
           <t>GLN (3), Туз Буби (4), PVL (7), levdanskiy (8), Jane Marduk (8), Елена (10)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>Tyla, Zara Larsson</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>SHE DID IT AGAIN</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="18" t="n">
         <v>36</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="15" t="n">
         <v>36</v>
       </c>
-      <c r="G13" s="7" t="n">
+      <c r="G13" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="18" t="inlineStr">
         <is>
           <t>80%</t>
         </is>
       </c>
-      <c r="I13" s="7" t="n">
+      <c r="I13" s="18" t="n">
         <v>3.75</v>
       </c>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="J13" s="18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="K13" s="17" t="inlineStr">
         <is>
           <t>PVL (3), Туз Буби (7), Imants (8), Елена (9), ТЁМА С. 🦂 (9), Ильдус (10), GLN (11), Jane Marduk (11)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Сергей Лазарев, Полина Гагарина</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Хэппи Энд</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="19" t="n">
         <v>33</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="G14" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="19" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
       </c>
-      <c r="I14" s="4" t="n">
+      <c r="I14" s="19" t="n">
         <v>5.5</v>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J14" s="19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K14" s="14" t="inlineStr">
         <is>
           <t>levdanskiy (3), Jane Marduk (4), Ильдус (6), Imants (9), ТЁМА С. 🦂 (10)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Madonna</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>Love Sensation</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="18" t="n">
         <v>14</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="18" t="n">
         <v>29</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="G15" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="18" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
       </c>
-      <c r="I15" s="7" t="n">
+      <c r="I15" s="18" t="n">
         <v>6.04</v>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J15" s="18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>ТЁМА С. 🦂 (2), Ильдус (4), Туз Буби (6), PVL (11)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>Dave, Tems</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Raindance</t>
         </is>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="12" t="n">
         <v>29</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="G16" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H16" s="19" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
       </c>
-      <c r="I16" s="4" t="n">
+      <c r="I16" s="19" t="n">
         <v>4.67</v>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J16" s="19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K16" s="14" t="inlineStr">
         <is>
           <t>Ильдус (2), Imants (3), GLN (10), Linh (10), Елена (12)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="5" t="n">
+      <c r="A17" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Madison Beer</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>lovergirl</t>
         </is>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="18" t="n">
         <v>16</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E17" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" s="15" t="n">
         <v>29</v>
       </c>
-      <c r="G17" s="7" t="n">
+      <c r="G17" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="18" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
       </c>
-      <c r="I17" s="7" t="n">
+      <c r="I17" s="18" t="n">
         <v>5.83</v>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J17" s="18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t>Linh (2), Imants (4), Ильдус (9), Jane Marduk (9)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>HOLLYFLAME</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Тону</t>
         </is>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="F18" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="G18" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H18" s="19" t="inlineStr">
         <is>
           <t>60%</t>
         </is>
       </c>
-      <c r="I18" s="4" t="n">
+      <c r="I18" s="19" t="n">
         <v>3.75</v>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="J18" s="19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K18" s="14" t="inlineStr">
         <is>
           <t>Imants (2), GLN (8), Linh (8), levdanskiy (10), Ильдус (11), PVL (12)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Dara</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>Bangaranga</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="E19" s="7" t="n">
+      <c r="E19" s="18" t="n">
         <v>23</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="15" t="n">
         <v>23</v>
       </c>
-      <c r="G19" s="7" t="n">
+      <c r="G19" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="18" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
       </c>
-      <c r="I19" s="7" t="n">
+      <c r="I19" s="18" t="n">
         <v>3.83</v>
       </c>
-      <c r="J19" s="7" t="inlineStr">
+      <c r="J19" s="18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="K19" s="17" t="inlineStr">
         <is>
           <t>ТЁМА С. 🦂 (7), GLN (7), Елена (8), PVL (8), levdanskiy (12)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>SAYAN</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>Мальборо</t>
         </is>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="D20" s="19" t="n">
         <v>19</v>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E20" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="F20" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="G20" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="19" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="I20" s="4" t="n">
+      <c r="I20" s="19" t="n">
         <v>3.89</v>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="J20" s="19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K20" s="14" t="inlineStr">
         <is>
           <t>GLN (4), PVL (9), Туз Буби (12)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="5" t="n">
+      <c r="A21" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>Ваня Дмитриенко</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>След</t>
         </is>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D21" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="E21" s="7" t="n">
+      <c r="E21" s="18" t="n">
         <v>13</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="G21" s="7" t="n">
+      <c r="G21" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H21" s="18" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
       </c>
-      <c r="I21" s="7" t="n">
+      <c r="I21" s="18" t="n">
         <v>2.71</v>
       </c>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="J21" s="18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K21" s="6" t="inlineStr">
+      <c r="K21" s="17" t="inlineStr">
         <is>
           <t>Елена (7), levdanskiy (9), ТЁМА С. 🦂 (11), Linh (12)</t>
         </is>
@@ -1469,7 +2085,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1496,1179 +2112,1179 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Место</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Исполнитель</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Песня</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>GLN</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Imants</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Jane Marduk</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Linh</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>PVL</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>levdanskiy</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Елена</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>Ильдус</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="11" t="inlineStr">
         <is>
           <t>ТЁМА С. 🦂</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="11" t="inlineStr">
         <is>
           <t>Туз Буби</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="11" t="inlineStr">
         <is>
           <t>Итог (Hit-Maker)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="11" t="inlineStr">
         <is>
           <t>Итог (Линейный)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Linda Lampenius &amp; Pete Parkkonen</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
         <is>
           <t>Liekinheitin</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>1 (15б)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>10 (3б)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>5 (8б)</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>6 (7б)</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="H2" s="19" t="inlineStr"/>
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>2 (12б)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>11 (2б)</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="12" t="inlineStr">
         <is>
           <t>5 (8б)</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="12" t="inlineStr">
         <is>
           <t>8 (5б)</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" s="12" t="inlineStr">
         <is>
           <t>2 (12б)</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="N2" s="12" t="n">
         <v>72</v>
       </c>
-      <c r="O2" s="4" t="n">
+      <c r="O2" s="19" t="n">
         <v>67</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>Taylor Swift</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>I Knew It, I Knew You</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="D3" s="18" t="inlineStr"/>
+      <c r="E3" s="21" t="inlineStr">
         <is>
           <t>1 (15б)</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="F3" s="18" t="inlineStr"/>
+      <c r="G3" s="21" t="inlineStr">
         <is>
           <t>1 (15б)</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr"/>
+      <c r="I3" s="15" t="inlineStr">
         <is>
           <t>6 (7б)</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" s="15" t="inlineStr">
         <is>
           <t>3 (10б)</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K3" s="15" t="inlineStr">
         <is>
           <t>12 (1б)</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L3" s="15" t="inlineStr">
         <is>
           <t>3 (10б)</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="M3" s="15" t="inlineStr">
         <is>
           <t>3 (10б)</t>
         </is>
       </c>
-      <c r="N3" s="5" t="n">
+      <c r="N3" s="15" t="n">
         <v>68</v>
       </c>
-      <c r="O3" s="7" t="n">
+      <c r="O3" s="18" t="n">
         <v>62</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>BLACKPINK</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>JUMP</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr"/>
+      <c r="E4" s="19" t="inlineStr"/>
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>1 (15б)</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="12" t="inlineStr">
         <is>
           <t>11 (2б)</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="H4" s="21" t="inlineStr">
         <is>
           <t>1 (15б)</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="I4" s="19" t="inlineStr"/>
+      <c r="J4" s="12" t="inlineStr">
         <is>
           <t>5 (8б)</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="12" t="inlineStr">
         <is>
           <t>8 (5б)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L4" s="12" t="inlineStr">
         <is>
           <t>5 (8б)</t>
         </is>
       </c>
-      <c r="M4" s="8" t="inlineStr">
+      <c r="M4" s="21" t="inlineStr">
         <is>
           <t>1 (15б)</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="N4" s="12" t="n">
         <v>68</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="O4" s="19" t="n">
         <v>59</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>BTS</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>SWIM</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>12 (1б)</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>11 (2б)</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>7 (6б)</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>9 (4б)</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>2 (12б)</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="15" t="inlineStr">
         <is>
           <t>5 (8б)</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="15" t="inlineStr">
         <is>
           <t>6 (7б)</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="15" t="inlineStr">
         <is>
           <t>3 (10б)</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="L5" s="18" t="inlineStr"/>
+      <c r="M5" s="15" t="inlineStr">
         <is>
           <t>8 (5б)</t>
         </is>
       </c>
-      <c r="N5" s="5" t="n">
+      <c r="N5" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="O5" s="7" t="n">
+      <c r="O5" s="18" t="n">
         <v>54</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>Olivia Rodrigo</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>drop dead</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>5 (8б)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>5 (8б)</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="F6" s="19" t="inlineStr"/>
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>4 (9б)</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>10 (3б)</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="I6" s="19" t="inlineStr"/>
+      <c r="J6" s="19" t="inlineStr"/>
+      <c r="K6" s="12" t="inlineStr">
         <is>
           <t>7 (6б)</t>
         </is>
       </c>
-      <c r="L6" s="8" t="inlineStr">
+      <c r="L6" s="21" t="inlineStr">
         <is>
           <t>1 (15б)</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M6" s="12" t="inlineStr">
         <is>
           <t>9 (4б)</t>
         </is>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="N6" s="12" t="n">
         <v>53</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="O6" s="19" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Sal Da Vinci</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>Per sempre sì</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr"/>
+      <c r="E7" s="18" t="inlineStr"/>
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>3 (10б)</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>3 (10б)</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="H7" s="18" t="inlineStr"/>
+      <c r="I7" s="15" t="inlineStr">
         <is>
           <t>4 (9б)</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>1 (15б)</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr"/>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="K7" s="18" t="inlineStr"/>
+      <c r="L7" s="15" t="inlineStr">
         <is>
           <t>4 (9б)</t>
         </is>
       </c>
-      <c r="M7" s="7" t="inlineStr"/>
-      <c r="N7" s="5" t="n">
+      <c r="M7" s="18" t="inlineStr"/>
+      <c r="N7" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="O7" s="7" t="n">
+      <c r="O7" s="18" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>By Индия, Xcho, МОТ</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Шадэ</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>6 (7б)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>6 (7б)</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>10 (3б)</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>7 (6б)</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>5 (8б)</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr">
         <is>
           <t>11 (2б)</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>2 (12б)</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr"/>
-      <c r="L8" s="4" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="K8" s="19" t="inlineStr"/>
+      <c r="L8" s="19" t="inlineStr"/>
+      <c r="M8" s="12" t="inlineStr">
         <is>
           <t>11 (2б)</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="N8" s="12" t="n">
         <v>47</v>
       </c>
-      <c r="O8" s="4" t="n">
+      <c r="O8" s="19" t="n">
         <v>46</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Alexandra Căpitănescu</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>Choke Me</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>2 (12б)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>12 (1б)</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>6 (7б)</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>5 (8б)</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="H9" s="18" t="inlineStr"/>
+      <c r="I9" s="15" t="inlineStr">
         <is>
           <t>7 (6б)</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr"/>
-      <c r="K9" s="7" t="inlineStr"/>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="J9" s="18" t="inlineStr"/>
+      <c r="K9" s="18" t="inlineStr"/>
+      <c r="L9" s="15" t="inlineStr">
         <is>
           <t>6 (7б)</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="M9" s="15" t="inlineStr">
         <is>
           <t>10 (3б)</t>
         </is>
       </c>
-      <c r="N9" s="5" t="n">
+      <c r="N9" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="O9" s="7" t="n">
+      <c r="O9" s="18" t="n">
         <v>43</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Егор Крид, ARTIK &amp; ASTI</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>KARMA</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>9 (4б)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>7 (6б)</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>12 (1б)</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="19" t="inlineStr"/>
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>4 (9б)</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
+      <c r="I10" s="21" t="inlineStr">
         <is>
           <t>1 (15б)</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>4 (9б)</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr"/>
-      <c r="L10" s="4" t="inlineStr"/>
-      <c r="M10" s="4" t="inlineStr"/>
-      <c r="N10" s="2" t="n">
+      <c r="K10" s="19" t="inlineStr"/>
+      <c r="L10" s="19" t="inlineStr"/>
+      <c r="M10" s="19" t="inlineStr"/>
+      <c r="N10" s="12" t="n">
         <v>44</v>
       </c>
-      <c r="O10" s="4" t="n">
+      <c r="O10" s="19" t="n">
         <v>41</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>KATSEYE</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>PINKY UP</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr"/>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr"/>
+      <c r="E11" s="18" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>2 (12б)</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="G11" s="18" t="inlineStr"/>
+      <c r="H11" s="15" t="inlineStr">
         <is>
           <t>6 (7б)</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr"/>
-      <c r="J11" s="7" t="inlineStr"/>
-      <c r="K11" s="8" t="inlineStr">
+      <c r="I11" s="18" t="inlineStr"/>
+      <c r="J11" s="18" t="inlineStr"/>
+      <c r="K11" s="21" t="inlineStr">
         <is>
           <t>1 (15б)</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="L11" s="15" t="inlineStr">
         <is>
           <t>12 (1б)</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="M11" s="15" t="inlineStr">
         <is>
           <t>5 (8б)</t>
         </is>
       </c>
-      <c r="N11" s="5" t="n">
+      <c r="N11" s="15" t="n">
         <v>43</v>
       </c>
-      <c r="O11" s="7" t="n">
+      <c r="O11" s="18" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>BEARWOLF</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Феникс</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>3 (10б)</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr"/>
+      <c r="F12" s="12" t="inlineStr">
         <is>
           <t>8 (5б)</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="19" t="inlineStr"/>
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>7 (6б)</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="12" t="inlineStr">
         <is>
           <t>8 (5б)</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" s="12" t="inlineStr">
         <is>
           <t>10 (3б)</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr"/>
-      <c r="L12" s="4" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="K12" s="19" t="inlineStr"/>
+      <c r="L12" s="19" t="inlineStr"/>
+      <c r="M12" s="12" t="inlineStr">
         <is>
           <t>4 (9б)</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="N12" s="12" t="n">
         <v>38</v>
       </c>
-      <c r="O12" s="4" t="n">
+      <c r="O12" s="19" t="n">
         <v>38</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>Tyla, Zara Larsson</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>SHE DID IT AGAIN</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>11 (2б)</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>8 (5б)</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="15" t="inlineStr">
         <is>
           <t>11 (2б)</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="G13" s="18" t="inlineStr"/>
+      <c r="H13" s="15" t="inlineStr">
         <is>
           <t>3 (10б)</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr"/>
+      <c r="J13" s="15" t="inlineStr">
         <is>
           <t>9 (4б)</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K13" s="15" t="inlineStr">
         <is>
           <t>10 (3б)</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="L13" s="15" t="inlineStr">
         <is>
           <t>9 (4б)</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="M13" s="15" t="inlineStr">
         <is>
           <t>7 (6б)</t>
         </is>
       </c>
-      <c r="N13" s="5" t="n">
+      <c r="N13" s="15" t="n">
         <v>36</v>
       </c>
-      <c r="O13" s="7" t="n">
+      <c r="O13" s="18" t="n">
         <v>36</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Сергей Лазарев, Полина Гагарина</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Хэппи Энд</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr"/>
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>9 (4б)</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F14" s="12" t="inlineStr">
         <is>
           <t>4 (9б)</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr"/>
-      <c r="H14" s="4" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="G14" s="19" t="inlineStr"/>
+      <c r="H14" s="19" t="inlineStr"/>
+      <c r="I14" s="12" t="inlineStr">
         <is>
           <t>3 (10б)</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="J14" s="19" t="inlineStr"/>
+      <c r="K14" s="12" t="inlineStr">
         <is>
           <t>6 (7б)</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L14" s="12" t="inlineStr">
         <is>
           <t>10 (3б)</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="2" t="n">
+      <c r="M14" s="19" t="inlineStr"/>
+      <c r="N14" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="O14" s="4" t="n">
+      <c r="O14" s="19" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Madonna</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>Love Sensation</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr"/>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr"/>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="D15" s="18" t="inlineStr"/>
+      <c r="E15" s="18" t="inlineStr"/>
+      <c r="F15" s="18" t="inlineStr"/>
+      <c r="G15" s="18" t="inlineStr"/>
+      <c r="H15" s="15" t="inlineStr">
         <is>
           <t>11 (2б)</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr"/>
-      <c r="J15" s="7" t="inlineStr"/>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="I15" s="18" t="inlineStr"/>
+      <c r="J15" s="18" t="inlineStr"/>
+      <c r="K15" s="15" t="inlineStr">
         <is>
           <t>4 (9б)</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="L15" s="15" t="inlineStr">
         <is>
           <t>2 (12б)</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="M15" s="15" t="inlineStr">
         <is>
           <t>6 (7б)</t>
         </is>
       </c>
-      <c r="N15" s="5" t="n">
+      <c r="N15" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="O15" s="7" t="n">
+      <c r="O15" s="18" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>Dave, Tems</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Raindance</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>10 (3б)</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="12" t="inlineStr">
         <is>
           <t>3 (10б)</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="F16" s="19" t="inlineStr"/>
+      <c r="G16" s="12" t="inlineStr">
         <is>
           <t>10 (3б)</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="H16" s="19" t="inlineStr"/>
+      <c r="I16" s="19" t="inlineStr"/>
+      <c r="J16" s="12" t="inlineStr">
         <is>
           <t>12 (1б)</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K16" s="12" t="inlineStr">
         <is>
           <t>2 (12б)</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="2" t="n">
+      <c r="L16" s="19" t="inlineStr"/>
+      <c r="M16" s="19" t="inlineStr"/>
+      <c r="N16" s="12" t="n">
         <v>29</v>
       </c>
-      <c r="O16" s="4" t="n">
+      <c r="O16" s="19" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="5" t="n">
+      <c r="A17" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Madison Beer</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>lovergirl</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr"/>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="D17" s="18" t="inlineStr"/>
+      <c r="E17" s="15" t="inlineStr">
         <is>
           <t>4 (9б)</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="15" t="inlineStr">
         <is>
           <t>9 (4б)</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="15" t="inlineStr">
         <is>
           <t>2 (12б)</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr"/>
-      <c r="I17" s="7" t="inlineStr"/>
-      <c r="J17" s="7" t="inlineStr"/>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="H17" s="18" t="inlineStr"/>
+      <c r="I17" s="18" t="inlineStr"/>
+      <c r="J17" s="18" t="inlineStr"/>
+      <c r="K17" s="15" t="inlineStr">
         <is>
           <t>9 (4б)</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr"/>
-      <c r="M17" s="7" t="inlineStr"/>
-      <c r="N17" s="5" t="n">
+      <c r="L17" s="18" t="inlineStr"/>
+      <c r="M17" s="18" t="inlineStr"/>
+      <c r="N17" s="15" t="n">
         <v>29</v>
       </c>
-      <c r="O17" s="7" t="n">
+      <c r="O17" s="18" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>HOLLYFLAME</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Тону</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>8 (5б)</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="12" t="inlineStr">
         <is>
           <t>2 (12б)</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="F18" s="19" t="inlineStr"/>
+      <c r="G18" s="12" t="inlineStr">
         <is>
           <t>8 (5б)</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" s="12" t="inlineStr">
         <is>
           <t>12 (1б)</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I18" s="12" t="inlineStr">
         <is>
           <t>10 (3б)</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="J18" s="19" t="inlineStr"/>
+      <c r="K18" s="12" t="inlineStr">
         <is>
           <t>11 (2б)</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="2" t="n">
+      <c r="L18" s="19" t="inlineStr"/>
+      <c r="M18" s="19" t="inlineStr"/>
+      <c r="N18" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="O18" s="4" t="n">
+      <c r="O18" s="19" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Dara</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>Bangaranga</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>7 (6б)</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr"/>
-      <c r="F19" s="7" t="inlineStr"/>
-      <c r="G19" s="7" t="inlineStr"/>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="E19" s="18" t="inlineStr"/>
+      <c r="F19" s="18" t="inlineStr"/>
+      <c r="G19" s="18" t="inlineStr"/>
+      <c r="H19" s="15" t="inlineStr">
         <is>
           <t>8 (5б)</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I19" s="15" t="inlineStr">
         <is>
           <t>12 (1б)</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="J19" s="15" t="inlineStr">
         <is>
           <t>8 (5б)</t>
         </is>
       </c>
-      <c r="K19" s="7" t="inlineStr"/>
-      <c r="L19" s="5" t="inlineStr">
+      <c r="K19" s="18" t="inlineStr"/>
+      <c r="L19" s="15" t="inlineStr">
         <is>
           <t>7 (6б)</t>
         </is>
       </c>
-      <c r="M19" s="7" t="inlineStr"/>
-      <c r="N19" s="5" t="n">
+      <c r="M19" s="18" t="inlineStr"/>
+      <c r="N19" s="15" t="n">
         <v>23</v>
       </c>
-      <c r="O19" s="7" t="n">
+      <c r="O19" s="18" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>SAYAN</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>Мальборо</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>4 (9б)</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr"/>
-      <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="E20" s="19" t="inlineStr"/>
+      <c r="F20" s="19" t="inlineStr"/>
+      <c r="G20" s="19" t="inlineStr"/>
+      <c r="H20" s="12" t="inlineStr">
         <is>
           <t>9 (4б)</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr"/>
-      <c r="J20" s="4" t="inlineStr"/>
-      <c r="K20" s="4" t="inlineStr"/>
-      <c r="L20" s="4" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="I20" s="19" t="inlineStr"/>
+      <c r="J20" s="19" t="inlineStr"/>
+      <c r="K20" s="19" t="inlineStr"/>
+      <c r="L20" s="19" t="inlineStr"/>
+      <c r="M20" s="12" t="inlineStr">
         <is>
           <t>12 (1б)</t>
         </is>
       </c>
-      <c r="N20" s="2" t="n">
+      <c r="N20" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="O20" s="4" t="n">
+      <c r="O20" s="19" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="5" t="n">
+      <c r="A21" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>Ваня Дмитриенко</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>След</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr"/>
-      <c r="E21" s="7" t="inlineStr"/>
-      <c r="F21" s="7" t="inlineStr"/>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="D21" s="18" t="inlineStr"/>
+      <c r="E21" s="18" t="inlineStr"/>
+      <c r="F21" s="18" t="inlineStr"/>
+      <c r="G21" s="15" t="inlineStr">
         <is>
           <t>12 (1б)</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr"/>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="H21" s="18" t="inlineStr"/>
+      <c r="I21" s="15" t="inlineStr">
         <is>
           <t>9 (4б)</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="J21" s="15" t="inlineStr">
         <is>
           <t>7 (6б)</t>
         </is>
       </c>
-      <c r="K21" s="7" t="inlineStr"/>
-      <c r="L21" s="5" t="inlineStr">
+      <c r="K21" s="18" t="inlineStr"/>
+      <c r="L21" s="15" t="inlineStr">
         <is>
           <t>11 (2б)</t>
         </is>
       </c>
-      <c r="M21" s="7" t="inlineStr"/>
-      <c r="N21" s="5" t="n">
+      <c r="M21" s="18" t="inlineStr"/>
+      <c r="N21" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="O21" s="7" t="n">
+      <c r="O21" s="18" t="n">
         <v>13</v>
       </c>
     </row>

</xml_diff>